<commit_message>
bug fix on abs units tubes and threshold tested
</commit_message>
<xml_diff>
--- a/config/tube_threshold_example.xlsx
+++ b/config/tube_threshold_example.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10703"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Projects\mbuty\config\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/francescopiscitelli/git_repos/mbuty/config/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0C415D98-2541-4973-9075-88E56EF36496}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7DB59DBF-5668-FD45-9980-A4506E2BD5D3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2850" yWindow="2210" windowWidth="19200" windowHeight="11170" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-34080" yWindow="6060" windowWidth="19200" windowHeight="11180" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet2" sheetId="2" r:id="rId1"/>
@@ -363,10 +363,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8D65F40D-01C7-4A1B-AA71-43574C5BB60D}">
-  <dimension ref="A1:D2"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <dimension ref="A1:F2"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A1">
         <v>1</v>
       </c>
@@ -379,8 +379,14 @@
       <c r="D1">
         <v>4</v>
       </c>
+      <c r="E1">
+        <v>13</v>
+      </c>
+      <c r="F1">
+        <v>14</v>
+      </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A2">
         <v>6000</v>
       </c>
@@ -392,6 +398,12 @@
       </c>
       <c r="D2">
         <v>7000</v>
+      </c>
+      <c r="E2">
+        <v>10000</v>
+      </c>
+      <c r="F2">
+        <v>8000</v>
       </c>
     </row>
   </sheetData>

</xml_diff>